<commit_message>
Organize project files and add build journal
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rcfab602a63b0448f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stardance request" sheetId="2" r:id="R07c1fecd159a4ad6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Self-funded" sheetId="3" r:id="R8c759bdc05734717"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rad225b7879d74157"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stardance request" sheetId="2" r:id="R54add96361d4429b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Self-funded" sheetId="3" r:id="Rd26c4f9547bd4218"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1108,7 +1108,7 @@
         <x:v>https://jlcpcb.com/</x:v>
       </x:c>
       <x:c r="I21" s="37" t="str">
-        <x:v>Fabricate using docs/pcb/Adapterboard-PTH.zip</x:v>
+        <x:v>Fabricate using PCB/Adapterboard-PTH.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="34" customHeight="1">
@@ -1138,7 +1138,7 @@
         <x:v>https://jlcpcb.com/</x:v>
       </x:c>
       <x:c r="I22" s="37" t="str">
-        <x:v>Fabricate using docs/pcb/Tunnelling-Amp.zip</x:v>
+        <x:v>Fabricate using PCB/Tunnelling-Amp.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="34" customHeight="1">

</xml_diff>